<commit_message>
Regenerate variant solutions.xlsx with apportioned %-impervious (SWMM-valid)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EaTiAK1cnJALW2TogbBHp
</commit_message>
<xml_diff>
--- a/results_combat/solution_balanced.xlsx
+++ b/results_combat/solution_balanced.xlsx
@@ -23257,7 +23257,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>53.1</v>
+        <v>52.7</v>
       </c>
       <c r="H7" t="n">
         <v>46.8</v>
@@ -23593,7 +23593,7 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>84.1699</v>
+        <v>83.6699</v>
       </c>
       <c r="H19" t="n">
         <v>15.8301</v>
@@ -24713,7 +24713,7 @@
         <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>65.63379999999999</v>
+        <v>65.13379999999999</v>
       </c>
       <c r="H59" t="n">
         <v>34.3662</v>
@@ -25189,7 +25189,7 @@
         <v>0</v>
       </c>
       <c r="G76" t="n">
-        <v>20.2301</v>
+        <v>19.7301</v>
       </c>
       <c r="H76" t="n">
         <v>79.76990000000001</v>
@@ -25357,7 +25357,7 @@
         <v>0</v>
       </c>
       <c r="G82" t="n">
-        <v>57.7922</v>
+        <v>57.2922</v>
       </c>
       <c r="H82" t="n">
         <v>42.2078</v>
@@ -25693,7 +25693,7 @@
         <v>0</v>
       </c>
       <c r="G94" t="n">
-        <v>52.8634</v>
+        <v>52.3634</v>
       </c>
       <c r="H94" t="n">
         <v>47.1366</v>
@@ -25721,7 +25721,7 @@
         <v>0</v>
       </c>
       <c r="G95" t="n">
-        <v>63.5731</v>
+        <v>63.0731</v>
       </c>
       <c r="H95" t="n">
         <v>36.4269</v>
@@ -25805,7 +25805,7 @@
         <v>0</v>
       </c>
       <c r="G98" t="n">
-        <v>65.7431</v>
+        <v>65.2431</v>
       </c>
       <c r="H98" t="n">
         <v>34.2569</v>
@@ -26284,7 +26284,7 @@
         <v>0</v>
       </c>
       <c r="H115" t="n">
-        <v>100</v>
+        <v>99.5</v>
       </c>
     </row>
     <row r="116">
@@ -26393,7 +26393,7 @@
         <v>0</v>
       </c>
       <c r="G119" t="n">
-        <v>46.0348</v>
+        <v>45.5348</v>
       </c>
       <c r="H119" t="n">
         <v>53.9652</v>
@@ -26449,7 +26449,7 @@
         <v>0</v>
       </c>
       <c r="G121" t="n">
-        <v>70.1863</v>
+        <v>69.6863</v>
       </c>
       <c r="H121" t="n">
         <v>29.8137</v>
@@ -26505,7 +26505,7 @@
         <v>0</v>
       </c>
       <c r="G123" t="n">
-        <v>56.9048</v>
+        <v>56.4048</v>
       </c>
       <c r="H123" t="n">
         <v>43.0952</v>
@@ -28341,7 +28341,7 @@
         <v>0</v>
       </c>
       <c r="C189" t="n">
-        <v>100</v>
+        <v>42.1658</v>
       </c>
       <c r="D189" t="n">
         <v>0</v>
@@ -28372,7 +28372,7 @@
         <v>0</v>
       </c>
       <c r="D190" t="n">
-        <v>100</v>
+        <v>17.1528</v>
       </c>
       <c r="E190" t="n">
         <v>0</v>
@@ -28717,7 +28717,7 @@
         <v>0</v>
       </c>
       <c r="G202" t="n">
-        <v>54.1935</v>
+        <v>53.6935</v>
       </c>
       <c r="H202" t="n">
         <v>45.8065</v>
@@ -28829,7 +28829,7 @@
         <v>0</v>
       </c>
       <c r="G206" t="n">
-        <v>47.5973</v>
+        <v>47.0973</v>
       </c>
       <c r="H206" t="n">
         <v>52.4027</v>
@@ -28941,7 +28941,7 @@
         <v>0</v>
       </c>
       <c r="G210" t="n">
-        <v>84.50700000000001</v>
+        <v>84.00700000000001</v>
       </c>
       <c r="H210" t="n">
         <v>15.493</v>
@@ -29122,7 +29122,7 @@
         </is>
       </c>
       <c r="B217" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="C217" t="n">
         <v>0</v>
@@ -29137,7 +29137,7 @@
         <v>0</v>
       </c>
       <c r="G217" t="n">
-        <v>39.9449</v>
+        <v>39.4449</v>
       </c>
       <c r="H217" t="n">
         <v>60.0551</v>
@@ -29165,7 +29165,7 @@
         <v>0</v>
       </c>
       <c r="G218" t="n">
-        <v>43.1599</v>
+        <v>42.6599</v>
       </c>
       <c r="H218" t="n">
         <v>56.8401</v>
@@ -29193,7 +29193,7 @@
         <v>0</v>
       </c>
       <c r="G219" t="n">
-        <v>65.16849999999999</v>
+        <v>64.66849999999999</v>
       </c>
       <c r="H219" t="n">
         <v>34.8315</v>
@@ -29557,7 +29557,7 @@
         <v>0</v>
       </c>
       <c r="G232" t="n">
-        <v>82.3322</v>
+        <v>81.8322</v>
       </c>
       <c r="H232" t="n">
         <v>17.6678</v>
@@ -30005,7 +30005,7 @@
         <v>0</v>
       </c>
       <c r="G248" t="n">
-        <v>56.9713</v>
+        <v>56.4713</v>
       </c>
       <c r="H248" t="n">
         <v>43.0287</v>
@@ -30033,7 +30033,7 @@
         <v>0</v>
       </c>
       <c r="G249" t="n">
-        <v>75.6549</v>
+        <v>75.1549</v>
       </c>
       <c r="H249" t="n">
         <v>24.3451</v>
@@ -30285,7 +30285,7 @@
         <v>0</v>
       </c>
       <c r="G258" t="n">
-        <v>58.4932</v>
+        <v>57.9932</v>
       </c>
       <c r="H258" t="n">
         <v>41.5068</v>
@@ -30313,7 +30313,7 @@
         <v>0</v>
       </c>
       <c r="G259" t="n">
-        <v>65.9513</v>
+        <v>65.4513</v>
       </c>
       <c r="H259" t="n">
         <v>34.0487</v>
@@ -30565,7 +30565,7 @@
         <v>0</v>
       </c>
       <c r="G268" t="n">
-        <v>53.6341</v>
+        <v>53.1341</v>
       </c>
       <c r="H268" t="n">
         <v>46.3659</v>
@@ -30957,7 +30957,7 @@
         <v>0</v>
       </c>
       <c r="G282" t="n">
-        <v>61.3674</v>
+        <v>60.8674</v>
       </c>
       <c r="H282" t="n">
         <v>38.6326</v>
@@ -31309,7 +31309,7 @@
         <v>0</v>
       </c>
       <c r="C295" t="n">
-        <v>100</v>
+        <v>44.8229</v>
       </c>
       <c r="D295" t="n">
         <v>0</v>
@@ -31405,7 +31405,7 @@
         <v>0</v>
       </c>
       <c r="G298" t="n">
-        <v>61.3169</v>
+        <v>60.8169</v>
       </c>
       <c r="H298" t="n">
         <v>38.6831</v>
@@ -31713,7 +31713,7 @@
         <v>0</v>
       </c>
       <c r="G309" t="n">
-        <v>58.5678</v>
+        <v>58.0678</v>
       </c>
       <c r="H309" t="n">
         <v>41.4322</v>
@@ -31741,7 +31741,7 @@
         <v>0</v>
       </c>
       <c r="G310" t="n">
-        <v>99.8353</v>
+        <v>99.5</v>
       </c>
       <c r="H310" t="n">
         <v>0</v>
@@ -31825,7 +31825,7 @@
         <v>0</v>
       </c>
       <c r="G313" t="n">
-        <v>68.4358</v>
+        <v>67.9358</v>
       </c>
       <c r="H313" t="n">
         <v>31.5642</v>
@@ -32049,7 +32049,7 @@
         <v>0</v>
       </c>
       <c r="G321" t="n">
-        <v>62.6301</v>
+        <v>62.1301</v>
       </c>
       <c r="H321" t="n">
         <v>37.3699</v>
@@ -33141,7 +33141,7 @@
         <v>0</v>
       </c>
       <c r="G360" t="n">
-        <v>57.2708</v>
+        <v>56.7708</v>
       </c>
       <c r="H360" t="n">
         <v>42.7292</v>
@@ -33253,7 +33253,7 @@
         <v>0</v>
       </c>
       <c r="G364" t="n">
-        <v>54.5455</v>
+        <v>54.0455</v>
       </c>
       <c r="H364" t="n">
         <v>45.4545</v>
@@ -33421,7 +33421,7 @@
         <v>0</v>
       </c>
       <c r="G370" t="n">
-        <v>47.1761</v>
+        <v>46.6761</v>
       </c>
       <c r="H370" t="n">
         <v>52.8239</v>
@@ -33505,7 +33505,7 @@
         <v>0</v>
       </c>
       <c r="G373" t="n">
-        <v>58.6111</v>
+        <v>58.1111</v>
       </c>
       <c r="H373" t="n">
         <v>41.3889</v>
@@ -33729,7 +33729,7 @@
         <v>0</v>
       </c>
       <c r="G381" t="n">
-        <v>50.7667</v>
+        <v>50.2667</v>
       </c>
       <c r="H381" t="n">
         <v>49.2333</v>
@@ -33757,7 +33757,7 @@
         <v>0</v>
       </c>
       <c r="G382" t="n">
-        <v>61.3647</v>
+        <v>60.8647</v>
       </c>
       <c r="H382" t="n">
         <v>38.6353</v>
@@ -33869,7 +33869,7 @@
         <v>0</v>
       </c>
       <c r="G386" t="n">
-        <v>46.3563</v>
+        <v>45.8563</v>
       </c>
       <c r="H386" t="n">
         <v>53.6437</v>
@@ -34289,7 +34289,7 @@
         <v>0</v>
       </c>
       <c r="G401" t="n">
-        <v>61.4286</v>
+        <v>60.9286</v>
       </c>
       <c r="H401" t="n">
         <v>38.5714</v>
@@ -34457,7 +34457,7 @@
         <v>0</v>
       </c>
       <c r="G407" t="n">
-        <v>42.268</v>
+        <v>41.768</v>
       </c>
       <c r="H407" t="n">
         <v>57.732</v>
@@ -34569,7 +34569,7 @@
         <v>0</v>
       </c>
       <c r="G411" t="n">
-        <v>70.48050000000001</v>
+        <v>69.98050000000001</v>
       </c>
       <c r="H411" t="n">
         <v>29.5195</v>
@@ -35997,7 +35997,7 @@
         <v>0</v>
       </c>
       <c r="G462" t="n">
-        <v>73.8019</v>
+        <v>73.3019</v>
       </c>
       <c r="H462" t="n">
         <v>26.1981</v>
@@ -36053,7 +36053,7 @@
         <v>0</v>
       </c>
       <c r="G464" t="n">
-        <v>47.1642</v>
+        <v>46.6642</v>
       </c>
       <c r="H464" t="n">
         <v>52.8358</v>
@@ -38072,7 +38072,7 @@
         <v>0</v>
       </c>
       <c r="H536" t="n">
-        <v>100</v>
+        <v>99.5</v>
       </c>
     </row>
     <row r="537">

</xml_diff>

<commit_message>
Validated results: rank variants by TOPSIS, select biodiverse submission
Evaluated baseline + 4 variants with SWMM on the 20 Aug-3 Sep 2018 storm
window. All benefit indicators move the right way vs baseline (flood/CSO/TSS
down, WWTP inflow and evaporation up). TOPSIS ranking over the seven
indicators: biodiverse (0.744) > balanced (0.611) > capture (0.446) >
thrifty (0.378).

solution_SUBMIT.xlsx = biodiverse: EUR 640,038 (98.5% of budget), biodiversity
600 m2, 299 interventions, 0 rule violations. Truncate (floor) written areas /
%-impervious so values never exceed the per-subcatchment caps.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EaTiAK1cnJALW2TogbBHp
</commit_message>
<xml_diff>
--- a/results_combat/solution_balanced.xlsx
+++ b/results_combat/solution_balanced.xlsx
@@ -743,7 +743,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>5.148</v>
+        <v>5.1479</v>
       </c>
     </row>
     <row r="12">
@@ -771,7 +771,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>5.4098</v>
+        <v>5.4097</v>
       </c>
     </row>
     <row r="13">
@@ -1107,7 +1107,7 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>1.8938</v>
+        <v>1.8937</v>
       </c>
     </row>
     <row r="25">
@@ -1247,7 +1247,7 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>2.6439</v>
+        <v>2.6438</v>
       </c>
     </row>
     <row r="30">
@@ -1555,7 +1555,7 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>3.5623</v>
+        <v>3.5622</v>
       </c>
     </row>
     <row r="41">
@@ -1695,7 +1695,7 @@
         <v>0</v>
       </c>
       <c r="H45" t="n">
-        <v>5.0743</v>
+        <v>5.0742</v>
       </c>
     </row>
     <row r="46">
@@ -1863,7 +1863,7 @@
         <v>0</v>
       </c>
       <c r="H51" t="n">
-        <v>2.3161</v>
+        <v>2.316</v>
       </c>
     </row>
     <row r="52">
@@ -2003,7 +2003,7 @@
         <v>0</v>
       </c>
       <c r="H56" t="n">
-        <v>5.0477</v>
+        <v>5.0476</v>
       </c>
     </row>
     <row r="57">
@@ -2059,7 +2059,7 @@
         <v>0</v>
       </c>
       <c r="H58" t="n">
-        <v>1.726</v>
+        <v>1.7259</v>
       </c>
     </row>
     <row r="59">
@@ -2087,7 +2087,7 @@
         <v>2</v>
       </c>
       <c r="H59" t="n">
-        <v>7.174</v>
+        <v>7.1739</v>
       </c>
     </row>
     <row r="60">
@@ -2143,7 +2143,7 @@
         <v>0</v>
       </c>
       <c r="H61" t="n">
-        <v>2.1287</v>
+        <v>2.1286</v>
       </c>
     </row>
     <row r="62">
@@ -2255,7 +2255,7 @@
         <v>0</v>
       </c>
       <c r="H65" t="n">
-        <v>2.3114</v>
+        <v>2.3113</v>
       </c>
     </row>
     <row r="66">
@@ -2367,7 +2367,7 @@
         <v>0</v>
       </c>
       <c r="H69" t="n">
-        <v>3.9156</v>
+        <v>3.9155</v>
       </c>
     </row>
     <row r="70">
@@ -2563,7 +2563,7 @@
         <v>2</v>
       </c>
       <c r="H76" t="n">
-        <v>48.9178</v>
+        <v>48.9177</v>
       </c>
     </row>
     <row r="77">
@@ -2703,7 +2703,7 @@
         <v>0</v>
       </c>
       <c r="H81" t="n">
-        <v>10.9553</v>
+        <v>10.9552</v>
       </c>
     </row>
     <row r="82">
@@ -2731,7 +2731,7 @@
         <v>2</v>
       </c>
       <c r="H82" t="n">
-        <v>11.4638</v>
+        <v>11.4637</v>
       </c>
     </row>
     <row r="83">
@@ -2787,7 +2787,7 @@
         <v>0</v>
       </c>
       <c r="H84" t="n">
-        <v>3.9385</v>
+        <v>3.9384</v>
       </c>
     </row>
     <row r="85">
@@ -3067,7 +3067,7 @@
         <v>2</v>
       </c>
       <c r="H94" t="n">
-        <v>12.6018</v>
+        <v>12.6017</v>
       </c>
     </row>
     <row r="95">
@@ -3095,7 +3095,7 @@
         <v>2</v>
       </c>
       <c r="H95" t="n">
-        <v>9.246600000000001</v>
+        <v>9.246499999999999</v>
       </c>
     </row>
     <row r="96">
@@ -3151,7 +3151,7 @@
         <v>0</v>
       </c>
       <c r="H97" t="n">
-        <v>4.7228</v>
+        <v>4.7227</v>
       </c>
     </row>
     <row r="98">
@@ -3487,7 +3487,7 @@
         <v>0</v>
       </c>
       <c r="H109" t="n">
-        <v>8.783200000000001</v>
+        <v>8.783099999999999</v>
       </c>
     </row>
     <row r="110">
@@ -3515,7 +3515,7 @@
         <v>0</v>
       </c>
       <c r="H110" t="n">
-        <v>6.4124</v>
+        <v>6.4123</v>
       </c>
     </row>
     <row r="111">
@@ -3767,7 +3767,7 @@
         <v>2</v>
       </c>
       <c r="H119" t="n">
-        <v>16.416</v>
+        <v>16.4159</v>
       </c>
     </row>
     <row r="120">
@@ -3851,7 +3851,7 @@
         <v>0</v>
       </c>
       <c r="H122" t="n">
-        <v>2.3123</v>
+        <v>2.3122</v>
       </c>
     </row>
     <row r="123">
@@ -3935,7 +3935,7 @@
         <v>0</v>
       </c>
       <c r="H125" t="n">
-        <v>1.8486</v>
+        <v>1.8485</v>
       </c>
     </row>
     <row r="126">
@@ -4019,7 +4019,7 @@
         <v>0</v>
       </c>
       <c r="H128" t="n">
-        <v>1.8237</v>
+        <v>1.8236</v>
       </c>
     </row>
     <row r="129">
@@ -4075,7 +4075,7 @@
         <v>0</v>
       </c>
       <c r="H130" t="n">
-        <v>3.0232</v>
+        <v>3.0231</v>
       </c>
     </row>
     <row r="131">
@@ -4103,7 +4103,7 @@
         <v>0</v>
       </c>
       <c r="H131" t="n">
-        <v>7.6653</v>
+        <v>7.6652</v>
       </c>
     </row>
     <row r="132">
@@ -4131,7 +4131,7 @@
         <v>0</v>
       </c>
       <c r="H132" t="n">
-        <v>5.1602</v>
+        <v>5.1601</v>
       </c>
     </row>
     <row r="133">
@@ -4215,7 +4215,7 @@
         <v>0</v>
       </c>
       <c r="H135" t="n">
-        <v>1.4832</v>
+        <v>1.4831</v>
       </c>
     </row>
     <row r="136">
@@ -4243,7 +4243,7 @@
         <v>0</v>
       </c>
       <c r="H136" t="n">
-        <v>2.1484</v>
+        <v>2.1483</v>
       </c>
     </row>
     <row r="137">
@@ -4523,7 +4523,7 @@
         <v>0</v>
       </c>
       <c r="H146" t="n">
-        <v>1.6719</v>
+        <v>1.6718</v>
       </c>
     </row>
     <row r="147">
@@ -4579,7 +4579,7 @@
         <v>0</v>
       </c>
       <c r="H148" t="n">
-        <v>2.4885</v>
+        <v>2.4884</v>
       </c>
     </row>
     <row r="149">
@@ -4663,7 +4663,7 @@
         <v>0</v>
       </c>
       <c r="H151" t="n">
-        <v>1.5379</v>
+        <v>1.5378</v>
       </c>
     </row>
     <row r="152">
@@ -5111,7 +5111,7 @@
         <v>0</v>
       </c>
       <c r="H167" t="n">
-        <v>1.4225</v>
+        <v>1.4224</v>
       </c>
     </row>
     <row r="168">
@@ -5447,7 +5447,7 @@
         <v>0</v>
       </c>
       <c r="H179" t="n">
-        <v>1.9181</v>
+        <v>1.918</v>
       </c>
     </row>
     <row r="180">
@@ -5475,7 +5475,7 @@
         <v>0</v>
       </c>
       <c r="H180" t="n">
-        <v>4.9633</v>
+        <v>4.9632</v>
       </c>
     </row>
     <row r="181">
@@ -5531,7 +5531,7 @@
         <v>0</v>
       </c>
       <c r="H182" t="n">
-        <v>3.5473</v>
+        <v>3.5472</v>
       </c>
     </row>
     <row r="183">
@@ -5923,7 +5923,7 @@
         <v>0</v>
       </c>
       <c r="H196" t="n">
-        <v>2.8499</v>
+        <v>2.8498</v>
       </c>
     </row>
     <row r="197">
@@ -6203,7 +6203,7 @@
         <v>2</v>
       </c>
       <c r="H206" t="n">
-        <v>13.4865</v>
+        <v>13.4864</v>
       </c>
     </row>
     <row r="207">
@@ -6343,7 +6343,7 @@
         <v>0</v>
       </c>
       <c r="H211" t="n">
-        <v>1.488</v>
+        <v>1.4879</v>
       </c>
     </row>
     <row r="212">
@@ -6399,7 +6399,7 @@
         <v>0</v>
       </c>
       <c r="H213" t="n">
-        <v>5.1339</v>
+        <v>5.1338</v>
       </c>
     </row>
     <row r="214">
@@ -6427,7 +6427,7 @@
         <v>0</v>
       </c>
       <c r="H214" t="n">
-        <v>4.7803</v>
+        <v>4.7802</v>
       </c>
     </row>
     <row r="215">
@@ -6493,7 +6493,7 @@
         </is>
       </c>
       <c r="B217" t="n">
-        <v>12.801</v>
+        <v>12.8009</v>
       </c>
       <c r="C217" t="n">
         <v>0</v>
@@ -6511,7 +6511,7 @@
         <v>2</v>
       </c>
       <c r="H217" t="n">
-        <v>25.6255</v>
+        <v>25.6254</v>
       </c>
     </row>
     <row r="218">
@@ -6539,7 +6539,7 @@
         <v>2</v>
       </c>
       <c r="H218" t="n">
-        <v>17.3573</v>
+        <v>17.3572</v>
       </c>
     </row>
     <row r="219">
@@ -6595,7 +6595,7 @@
         <v>0</v>
       </c>
       <c r="H220" t="n">
-        <v>3.2007</v>
+        <v>3.2006</v>
       </c>
     </row>
     <row r="221">
@@ -6651,7 +6651,7 @@
         <v>0</v>
       </c>
       <c r="H222" t="n">
-        <v>1.4392</v>
+        <v>1.4391</v>
       </c>
     </row>
     <row r="223">
@@ -6763,7 +6763,7 @@
         <v>0</v>
       </c>
       <c r="H226" t="n">
-        <v>1.8327</v>
+        <v>1.8326</v>
       </c>
     </row>
     <row r="227">
@@ -6931,7 +6931,7 @@
         <v>2</v>
       </c>
       <c r="H232" t="n">
-        <v>2.9404</v>
+        <v>2.9403</v>
       </c>
     </row>
     <row r="233">
@@ -7043,7 +7043,7 @@
         <v>0</v>
       </c>
       <c r="H236" t="n">
-        <v>1.7145</v>
+        <v>1.7144</v>
       </c>
     </row>
     <row r="237">
@@ -7379,7 +7379,7 @@
         <v>5</v>
       </c>
       <c r="H248" t="n">
-        <v>37.8966</v>
+        <v>37.8965</v>
       </c>
     </row>
     <row r="249">
@@ -7407,7 +7407,7 @@
         <v>5</v>
       </c>
       <c r="H249" t="n">
-        <v>18.5607</v>
+        <v>18.5606</v>
       </c>
     </row>
     <row r="250">
@@ -7575,7 +7575,7 @@
         <v>0</v>
       </c>
       <c r="H255" t="n">
-        <v>1.6073</v>
+        <v>1.6072</v>
       </c>
     </row>
     <row r="256">
@@ -7659,7 +7659,7 @@
         <v>5</v>
       </c>
       <c r="H258" t="n">
-        <v>34.3076</v>
+        <v>34.3075</v>
       </c>
     </row>
     <row r="259">
@@ -7687,7 +7687,7 @@
         <v>10</v>
       </c>
       <c r="H259" t="n">
-        <v>34.4916</v>
+        <v>34.4915</v>
       </c>
     </row>
     <row r="260">
@@ -7883,7 +7883,7 @@
         <v>0</v>
       </c>
       <c r="H266" t="n">
-        <v>2.0702</v>
+        <v>2.0701</v>
       </c>
     </row>
     <row r="267">
@@ -7939,7 +7939,7 @@
         <v>2</v>
       </c>
       <c r="H268" t="n">
-        <v>10.8914</v>
+        <v>10.8913</v>
       </c>
     </row>
     <row r="269">
@@ -8359,7 +8359,7 @@
         <v>0</v>
       </c>
       <c r="H283" t="n">
-        <v>1.4225</v>
+        <v>1.4224</v>
       </c>
     </row>
     <row r="284">
@@ -8387,7 +8387,7 @@
         <v>0</v>
       </c>
       <c r="H284" t="n">
-        <v>2.3003</v>
+        <v>2.3002</v>
       </c>
     </row>
     <row r="285">
@@ -8667,7 +8667,7 @@
         <v>0</v>
       </c>
       <c r="H294" t="n">
-        <v>7.2198</v>
+        <v>7.2197</v>
       </c>
     </row>
     <row r="295">
@@ -8680,7 +8680,7 @@
         <v>0</v>
       </c>
       <c r="C295" t="n">
-        <v>371.0466</v>
+        <v>371.0465</v>
       </c>
       <c r="D295" t="n">
         <v>0</v>
@@ -8891,7 +8891,7 @@
         <v>0</v>
       </c>
       <c r="H302" t="n">
-        <v>5.5018</v>
+        <v>5.5017</v>
       </c>
     </row>
     <row r="303">
@@ -9255,7 +9255,7 @@
         <v>0</v>
       </c>
       <c r="H315" t="n">
-        <v>19.6821</v>
+        <v>19.682</v>
       </c>
     </row>
     <row r="316">
@@ -9283,7 +9283,7 @@
         <v>0</v>
       </c>
       <c r="H316" t="n">
-        <v>2.8934</v>
+        <v>2.8933</v>
       </c>
     </row>
     <row r="317">
@@ -9311,7 +9311,7 @@
         <v>0</v>
       </c>
       <c r="H317" t="n">
-        <v>5.0652</v>
+        <v>5.0651</v>
       </c>
     </row>
     <row r="318">
@@ -9423,7 +9423,7 @@
         <v>10</v>
       </c>
       <c r="H321" t="n">
-        <v>40.0724</v>
+        <v>40.0723</v>
       </c>
     </row>
     <row r="322">
@@ -9451,7 +9451,7 @@
         <v>0</v>
       </c>
       <c r="H322" t="n">
-        <v>3.1782</v>
+        <v>3.1781</v>
       </c>
     </row>
     <row r="323">
@@ -9479,7 +9479,7 @@
         <v>0</v>
       </c>
       <c r="H323" t="n">
-        <v>2.7184</v>
+        <v>2.7183</v>
       </c>
     </row>
     <row r="324">
@@ -9619,7 +9619,7 @@
         <v>0</v>
       </c>
       <c r="H328" t="n">
-        <v>2.0039</v>
+        <v>2.0038</v>
       </c>
     </row>
     <row r="329">
@@ -9647,7 +9647,7 @@
         <v>0</v>
       </c>
       <c r="H329" t="n">
-        <v>4.6767</v>
+        <v>4.6766</v>
       </c>
     </row>
     <row r="330">
@@ -9815,7 +9815,7 @@
         <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>1.9035</v>
+        <v>1.9034</v>
       </c>
     </row>
     <row r="336">
@@ -9955,7 +9955,7 @@
         <v>0</v>
       </c>
       <c r="H340" t="n">
-        <v>1.8995</v>
+        <v>1.8994</v>
       </c>
     </row>
     <row r="341">
@@ -9983,7 +9983,7 @@
         <v>0</v>
       </c>
       <c r="H341" t="n">
-        <v>3.146</v>
+        <v>3.1459</v>
       </c>
     </row>
     <row r="342">
@@ -10095,7 +10095,7 @@
         <v>0</v>
       </c>
       <c r="H345" t="n">
-        <v>6.7187</v>
+        <v>6.7186</v>
       </c>
     </row>
     <row r="346">
@@ -10207,7 +10207,7 @@
         <v>0</v>
       </c>
       <c r="H349" t="n">
-        <v>1.5917</v>
+        <v>1.5916</v>
       </c>
     </row>
     <row r="350">
@@ -10235,7 +10235,7 @@
         <v>0</v>
       </c>
       <c r="H350" t="n">
-        <v>1.7129</v>
+        <v>1.7128</v>
       </c>
     </row>
     <row r="351">
@@ -10319,7 +10319,7 @@
         <v>0</v>
       </c>
       <c r="H353" t="n">
-        <v>2.6626</v>
+        <v>2.6625</v>
       </c>
     </row>
     <row r="354">
@@ -10347,7 +10347,7 @@
         <v>0</v>
       </c>
       <c r="H354" t="n">
-        <v>2.7402</v>
+        <v>2.7401</v>
       </c>
     </row>
     <row r="355">
@@ -10515,7 +10515,7 @@
         <v>5</v>
       </c>
       <c r="H360" t="n">
-        <v>36.4346</v>
+        <v>36.4345</v>
       </c>
     </row>
     <row r="361">
@@ -10655,7 +10655,7 @@
         <v>0</v>
       </c>
       <c r="H365" t="n">
-        <v>8.4171</v>
+        <v>8.417</v>
       </c>
     </row>
     <row r="366">
@@ -10767,7 +10767,7 @@
         <v>0</v>
       </c>
       <c r="H369" t="n">
-        <v>3.7808</v>
+        <v>3.7807</v>
       </c>
     </row>
     <row r="370">
@@ -10851,7 +10851,7 @@
         <v>0</v>
       </c>
       <c r="H372" t="n">
-        <v>9.0792</v>
+        <v>9.0791</v>
       </c>
     </row>
     <row r="373">
@@ -11047,7 +11047,7 @@
         <v>0</v>
       </c>
       <c r="H379" t="n">
-        <v>2.9054</v>
+        <v>2.9053</v>
       </c>
     </row>
     <row r="380">
@@ -11075,7 +11075,7 @@
         <v>0</v>
       </c>
       <c r="H380" t="n">
-        <v>7.8034</v>
+        <v>7.8033</v>
       </c>
     </row>
     <row r="381">
@@ -11103,7 +11103,7 @@
         <v>5</v>
       </c>
       <c r="H381" t="n">
-        <v>35.8541</v>
+        <v>35.854</v>
       </c>
     </row>
     <row r="382">
@@ -11131,7 +11131,7 @@
         <v>10</v>
       </c>
       <c r="H382" t="n">
-        <v>48.2246</v>
+        <v>48.2245</v>
       </c>
     </row>
     <row r="383">
@@ -11243,7 +11243,7 @@
         <v>2</v>
       </c>
       <c r="H386" t="n">
-        <v>15.5779</v>
+        <v>15.5778</v>
       </c>
     </row>
     <row r="387">
@@ -11327,7 +11327,7 @@
         <v>0</v>
       </c>
       <c r="H389" t="n">
-        <v>2.3728</v>
+        <v>2.3727</v>
       </c>
     </row>
     <row r="390">
@@ -11383,7 +11383,7 @@
         <v>0</v>
       </c>
       <c r="H391" t="n">
-        <v>2.383</v>
+        <v>2.3829</v>
       </c>
     </row>
     <row r="392">
@@ -11467,7 +11467,7 @@
         <v>0</v>
       </c>
       <c r="H394" t="n">
-        <v>2.8407</v>
+        <v>2.8406</v>
       </c>
     </row>
     <row r="395">
@@ -11551,7 +11551,7 @@
         <v>0</v>
       </c>
       <c r="H397" t="n">
-        <v>4.0087</v>
+        <v>4.0086</v>
       </c>
     </row>
     <row r="398">
@@ -11579,7 +11579,7 @@
         <v>0</v>
       </c>
       <c r="H398" t="n">
-        <v>1.8465</v>
+        <v>1.8464</v>
       </c>
     </row>
     <row r="399">
@@ -11607,7 +11607,7 @@
         <v>0</v>
       </c>
       <c r="H399" t="n">
-        <v>2.3405</v>
+        <v>2.3404</v>
       </c>
     </row>
     <row r="400">
@@ -11663,7 +11663,7 @@
         <v>4</v>
       </c>
       <c r="H401" t="n">
-        <v>15.8875</v>
+        <v>15.8874</v>
       </c>
     </row>
     <row r="402">
@@ -11747,7 +11747,7 @@
         <v>0</v>
       </c>
       <c r="H404" t="n">
-        <v>1.4564</v>
+        <v>1.4563</v>
       </c>
     </row>
     <row r="405">
@@ -11831,7 +11831,7 @@
         <v>3</v>
       </c>
       <c r="H407" t="n">
-        <v>26.3258</v>
+        <v>26.3257</v>
       </c>
     </row>
     <row r="408">
@@ -11887,7 +11887,7 @@
         <v>0</v>
       </c>
       <c r="H409" t="n">
-        <v>4.0147</v>
+        <v>4.0146</v>
       </c>
     </row>
     <row r="410">
@@ -11943,7 +11943,7 @@
         <v>3</v>
       </c>
       <c r="H411" t="n">
-        <v>7.5799</v>
+        <v>7.5798</v>
       </c>
     </row>
     <row r="412">
@@ -11971,7 +11971,7 @@
         <v>0</v>
       </c>
       <c r="H412" t="n">
-        <v>3.4854</v>
+        <v>3.4853</v>
       </c>
     </row>
     <row r="413">
@@ -11999,7 +11999,7 @@
         <v>0</v>
       </c>
       <c r="H413" t="n">
-        <v>9.097099999999999</v>
+        <v>9.097</v>
       </c>
     </row>
     <row r="414">
@@ -12363,7 +12363,7 @@
         <v>0</v>
       </c>
       <c r="H426" t="n">
-        <v>8.323700000000001</v>
+        <v>8.323600000000001</v>
       </c>
     </row>
     <row r="427">
@@ -12391,7 +12391,7 @@
         <v>0</v>
       </c>
       <c r="H427" t="n">
-        <v>4.3786</v>
+        <v>4.3785</v>
       </c>
     </row>
     <row r="428">
@@ -12587,7 +12587,7 @@
         <v>0</v>
       </c>
       <c r="H434" t="n">
-        <v>1.8317</v>
+        <v>1.8316</v>
       </c>
     </row>
     <row r="435">
@@ -12643,7 +12643,7 @@
         <v>0</v>
       </c>
       <c r="H436" t="n">
-        <v>3.3896</v>
+        <v>3.3895</v>
       </c>
     </row>
     <row r="437">
@@ -12671,7 +12671,7 @@
         <v>0</v>
       </c>
       <c r="H437" t="n">
-        <v>3.3333</v>
+        <v>3.3332</v>
       </c>
     </row>
     <row r="438">
@@ -12755,7 +12755,7 @@
         <v>0</v>
       </c>
       <c r="H440" t="n">
-        <v>5.0945</v>
+        <v>5.0944</v>
       </c>
     </row>
     <row r="441">
@@ -12783,7 +12783,7 @@
         <v>0</v>
       </c>
       <c r="H441" t="n">
-        <v>1.5346</v>
+        <v>1.5345</v>
       </c>
     </row>
     <row r="442">
@@ -12895,7 +12895,7 @@
         <v>0</v>
       </c>
       <c r="H445" t="n">
-        <v>3.6167</v>
+        <v>3.6166</v>
       </c>
     </row>
     <row r="446">
@@ -13175,7 +13175,7 @@
         <v>0</v>
       </c>
       <c r="H455" t="n">
-        <v>2.4207</v>
+        <v>2.4206</v>
       </c>
     </row>
     <row r="456">
@@ -13259,7 +13259,7 @@
         <v>0</v>
       </c>
       <c r="H458" t="n">
-        <v>1.6694</v>
+        <v>1.6693</v>
       </c>
     </row>
     <row r="459">
@@ -13287,7 +13287,7 @@
         <v>0</v>
       </c>
       <c r="H459" t="n">
-        <v>2.2424</v>
+        <v>2.2423</v>
       </c>
     </row>
     <row r="460">
@@ -13511,7 +13511,7 @@
         <v>0</v>
       </c>
       <c r="H467" t="n">
-        <v>3.1422</v>
+        <v>3.1421</v>
       </c>
     </row>
     <row r="468">
@@ -13623,7 +13623,7 @@
         <v>0</v>
       </c>
       <c r="H471" t="n">
-        <v>3.0137</v>
+        <v>3.0136</v>
       </c>
     </row>
     <row r="472">
@@ -13651,7 +13651,7 @@
         <v>0</v>
       </c>
       <c r="H472" t="n">
-        <v>14.6171</v>
+        <v>14.617</v>
       </c>
     </row>
     <row r="473">
@@ -13847,7 +13847,7 @@
         <v>0</v>
       </c>
       <c r="H479" t="n">
-        <v>6.2362</v>
+        <v>6.2361</v>
       </c>
     </row>
     <row r="480">
@@ -14155,7 +14155,7 @@
         <v>0</v>
       </c>
       <c r="H490" t="n">
-        <v>3.6008</v>
+        <v>3.6007</v>
       </c>
     </row>
     <row r="491">
@@ -14239,7 +14239,7 @@
         <v>0</v>
       </c>
       <c r="H493" t="n">
-        <v>7.1331</v>
+        <v>7.133</v>
       </c>
     </row>
     <row r="494">
@@ -14323,7 +14323,7 @@
         <v>0</v>
       </c>
       <c r="H496" t="n">
-        <v>3.7871</v>
+        <v>3.787</v>
       </c>
     </row>
     <row r="497">
@@ -14351,7 +14351,7 @@
         <v>0</v>
       </c>
       <c r="H497" t="n">
-        <v>1.9523</v>
+        <v>1.9522</v>
       </c>
     </row>
     <row r="498">
@@ -14967,7 +14967,7 @@
         <v>0</v>
       </c>
       <c r="H519" t="n">
-        <v>1.5621</v>
+        <v>1.562</v>
       </c>
     </row>
     <row r="520">
@@ -15051,7 +15051,7 @@
         <v>0</v>
       </c>
       <c r="H522" t="n">
-        <v>3.1882</v>
+        <v>3.1881</v>
       </c>
     </row>
     <row r="523">
@@ -15079,7 +15079,7 @@
         <v>0</v>
       </c>
       <c r="H523" t="n">
-        <v>2.893</v>
+        <v>2.8929</v>
       </c>
     </row>
     <row r="524">
@@ -15107,7 +15107,7 @@
         <v>0</v>
       </c>
       <c r="H524" t="n">
-        <v>2.5384</v>
+        <v>2.5383</v>
       </c>
     </row>
     <row r="525">
@@ -15163,7 +15163,7 @@
         <v>0</v>
       </c>
       <c r="H526" t="n">
-        <v>4.7164</v>
+        <v>4.7163</v>
       </c>
     </row>
     <row r="527">
@@ -15191,7 +15191,7 @@
         <v>0</v>
       </c>
       <c r="H527" t="n">
-        <v>9.2506</v>
+        <v>9.250500000000001</v>
       </c>
     </row>
     <row r="528">
@@ -15247,7 +15247,7 @@
         <v>0</v>
       </c>
       <c r="H529" t="n">
-        <v>2.9418</v>
+        <v>2.9417</v>
       </c>
     </row>
     <row r="530">
@@ -15303,7 +15303,7 @@
         <v>0</v>
       </c>
       <c r="H531" t="n">
-        <v>2.299</v>
+        <v>2.2989</v>
       </c>
     </row>
     <row r="532">
@@ -15387,7 +15387,7 @@
         <v>0</v>
       </c>
       <c r="H534" t="n">
-        <v>3.5461</v>
+        <v>3.546</v>
       </c>
     </row>
     <row r="535">
@@ -15415,7 +15415,7 @@
         <v>0</v>
       </c>
       <c r="H535" t="n">
-        <v>2.5965</v>
+        <v>2.5964</v>
       </c>
     </row>
     <row r="536">
@@ -15443,7 +15443,7 @@
         <v>0</v>
       </c>
       <c r="H536" t="n">
-        <v>2.9128</v>
+        <v>2.9127</v>
       </c>
     </row>
     <row r="537">
@@ -15499,7 +15499,7 @@
         <v>0</v>
       </c>
       <c r="H538" t="n">
-        <v>2.3081</v>
+        <v>2.308</v>
       </c>
     </row>
     <row r="539">
@@ -15527,7 +15527,7 @@
         <v>0</v>
       </c>
       <c r="H539" t="n">
-        <v>4.5537</v>
+        <v>4.5536</v>
       </c>
     </row>
     <row r="540">
@@ -23344,7 +23344,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>29.2398</v>
+        <v>29.2397</v>
       </c>
     </row>
     <row r="11">
@@ -23400,7 +23400,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>45.5446</v>
+        <v>45.5445</v>
       </c>
     </row>
     <row r="13">
@@ -23484,7 +23484,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>45.2555</v>
+        <v>45.2554</v>
       </c>
     </row>
     <row r="16">
@@ -23568,7 +23568,7 @@
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>34.6154</v>
+        <v>34.6153</v>
       </c>
     </row>
     <row r="19">
@@ -23593,7 +23593,7 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>83.6699</v>
+        <v>83.6698</v>
       </c>
       <c r="H19" t="n">
         <v>15.8301</v>
@@ -23652,7 +23652,7 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>35.9155</v>
+        <v>35.9154</v>
       </c>
     </row>
     <row r="22">
@@ -23708,7 +23708,7 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>21.2644</v>
+        <v>21.2643</v>
       </c>
     </row>
     <row r="24">
@@ -23792,7 +23792,7 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>21.2644</v>
+        <v>21.2643</v>
       </c>
     </row>
     <row r="27">
@@ -23848,7 +23848,7 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>42.5532</v>
+        <v>42.5531</v>
       </c>
     </row>
     <row r="29">
@@ -23904,7 +23904,7 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>89.0411</v>
+        <v>89.041</v>
       </c>
     </row>
     <row r="31">
@@ -23932,7 +23932,7 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>93.7107</v>
+        <v>93.7106</v>
       </c>
     </row>
     <row r="32">
@@ -23960,7 +23960,7 @@
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>31.5385</v>
+        <v>31.5384</v>
       </c>
     </row>
     <row r="33">
@@ -24072,7 +24072,7 @@
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>29.4872</v>
+        <v>29.4871</v>
       </c>
     </row>
     <row r="37">
@@ -24100,7 +24100,7 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>18.4783</v>
+        <v>18.4782</v>
       </c>
     </row>
     <row r="38">
@@ -24212,7 +24212,7 @@
         <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>19.6203</v>
+        <v>19.6202</v>
       </c>
     </row>
     <row r="42">
@@ -24324,7 +24324,7 @@
         <v>0</v>
       </c>
       <c r="H45" t="n">
-        <v>30.3887</v>
+        <v>30.3886</v>
       </c>
     </row>
     <row r="46">
@@ -24436,7 +24436,7 @@
         <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>62.6437</v>
+        <v>62.6436</v>
       </c>
     </row>
     <row r="50">
@@ -24576,7 +24576,7 @@
         <v>0</v>
       </c>
       <c r="H54" t="n">
-        <v>27.8689</v>
+        <v>27.8688</v>
       </c>
     </row>
     <row r="55">
@@ -24632,7 +24632,7 @@
         <v>0</v>
       </c>
       <c r="H56" t="n">
-        <v>55.5556</v>
+        <v>55.5555</v>
       </c>
     </row>
     <row r="57">
@@ -24716,7 +24716,7 @@
         <v>65.13379999999999</v>
       </c>
       <c r="H59" t="n">
-        <v>34.3662</v>
+        <v>34.3661</v>
       </c>
     </row>
     <row r="60">
@@ -24772,7 +24772,7 @@
         <v>0</v>
       </c>
       <c r="H61" t="n">
-        <v>24.8276</v>
+        <v>24.8275</v>
       </c>
     </row>
     <row r="62">
@@ -24828,7 +24828,7 @@
         <v>0</v>
       </c>
       <c r="H63" t="n">
-        <v>84.5865</v>
+        <v>84.5864</v>
       </c>
     </row>
     <row r="64">
@@ -24884,7 +24884,7 @@
         <v>0</v>
       </c>
       <c r="H65" t="n">
-        <v>23.9264</v>
+        <v>23.9263</v>
       </c>
     </row>
     <row r="66">
@@ -24996,7 +24996,7 @@
         <v>0</v>
       </c>
       <c r="H69" t="n">
-        <v>54.0984</v>
+        <v>54.0983</v>
       </c>
     </row>
     <row r="70">
@@ -25192,7 +25192,7 @@
         <v>19.7301</v>
       </c>
       <c r="H76" t="n">
-        <v>79.76990000000001</v>
+        <v>79.7698</v>
       </c>
     </row>
     <row r="77">
@@ -25245,7 +25245,7 @@
         <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>98.5577</v>
+        <v>98.55759999999999</v>
       </c>
       <c r="H78" t="n">
         <v>0</v>
@@ -25332,7 +25332,7 @@
         <v>0</v>
       </c>
       <c r="H81" t="n">
-        <v>55.1929</v>
+        <v>55.1928</v>
       </c>
     </row>
     <row r="82">
@@ -25360,7 +25360,7 @@
         <v>57.2922</v>
       </c>
       <c r="H82" t="n">
-        <v>42.2078</v>
+        <v>42.2077</v>
       </c>
     </row>
     <row r="83">
@@ -25668,7 +25668,7 @@
         <v>0</v>
       </c>
       <c r="H93" t="n">
-        <v>83.9117</v>
+        <v>83.91160000000001</v>
       </c>
     </row>
     <row r="94">
@@ -25696,7 +25696,7 @@
         <v>52.3634</v>
       </c>
       <c r="H94" t="n">
-        <v>47.1366</v>
+        <v>47.1365</v>
       </c>
     </row>
     <row r="95">
@@ -25721,7 +25721,7 @@
         <v>0</v>
       </c>
       <c r="G95" t="n">
-        <v>63.0731</v>
+        <v>63.073</v>
       </c>
       <c r="H95" t="n">
         <v>36.4269</v>
@@ -25752,7 +25752,7 @@
         <v>0</v>
       </c>
       <c r="H96" t="n">
-        <v>32.8829</v>
+        <v>32.8828</v>
       </c>
     </row>
     <row r="97">
@@ -25780,7 +25780,7 @@
         <v>0</v>
       </c>
       <c r="H97" t="n">
-        <v>33.7553</v>
+        <v>33.7552</v>
       </c>
     </row>
     <row r="98">
@@ -25805,7 +25805,7 @@
         <v>0</v>
       </c>
       <c r="G98" t="n">
-        <v>65.2431</v>
+        <v>65.24299999999999</v>
       </c>
       <c r="H98" t="n">
         <v>34.2569</v>
@@ -26088,7 +26088,7 @@
         <v>0</v>
       </c>
       <c r="H108" t="n">
-        <v>43.1953</v>
+        <v>43.1952</v>
       </c>
     </row>
     <row r="109">
@@ -26116,7 +26116,7 @@
         <v>0</v>
       </c>
       <c r="H109" t="n">
-        <v>56.4394</v>
+        <v>56.4393</v>
       </c>
     </row>
     <row r="110">
@@ -26144,7 +26144,7 @@
         <v>0</v>
       </c>
       <c r="H110" t="n">
-        <v>38.6525</v>
+        <v>38.6524</v>
       </c>
     </row>
     <row r="111">
@@ -26396,7 +26396,7 @@
         <v>45.5348</v>
       </c>
       <c r="H119" t="n">
-        <v>53.9652</v>
+        <v>53.9651</v>
       </c>
     </row>
     <row r="120">
@@ -26452,7 +26452,7 @@
         <v>69.6863</v>
       </c>
       <c r="H121" t="n">
-        <v>29.8137</v>
+        <v>29.8136</v>
       </c>
     </row>
     <row r="122">
@@ -26505,7 +26505,7 @@
         <v>0</v>
       </c>
       <c r="G123" t="n">
-        <v>56.4048</v>
+        <v>56.4047</v>
       </c>
       <c r="H123" t="n">
         <v>43.0952</v>
@@ -26620,7 +26620,7 @@
         <v>0</v>
       </c>
       <c r="H127" t="n">
-        <v>23.8411</v>
+        <v>23.841</v>
       </c>
     </row>
     <row r="128">
@@ -26704,7 +26704,7 @@
         <v>0</v>
       </c>
       <c r="H130" t="n">
-        <v>27.4194</v>
+        <v>27.4193</v>
       </c>
     </row>
     <row r="131">
@@ -26760,7 +26760,7 @@
         <v>0</v>
       </c>
       <c r="H132" t="n">
-        <v>58</v>
+        <v>57.9999</v>
       </c>
     </row>
     <row r="133">
@@ -26788,7 +26788,7 @@
         <v>0</v>
       </c>
       <c r="H133" t="n">
-        <v>52.6316</v>
+        <v>52.6315</v>
       </c>
     </row>
     <row r="134">
@@ -26816,7 +26816,7 @@
         <v>0</v>
       </c>
       <c r="H134" t="n">
-        <v>57.1429</v>
+        <v>57.1428</v>
       </c>
     </row>
     <row r="135">
@@ -26844,7 +26844,7 @@
         <v>0</v>
       </c>
       <c r="H135" t="n">
-        <v>32.0513</v>
+        <v>32.0512</v>
       </c>
     </row>
     <row r="136">
@@ -27152,7 +27152,7 @@
         <v>0</v>
       </c>
       <c r="H146" t="n">
-        <v>38.8889</v>
+        <v>38.8888</v>
       </c>
     </row>
     <row r="147">
@@ -27180,7 +27180,7 @@
         <v>0</v>
       </c>
       <c r="H147" t="n">
-        <v>35.4244</v>
+        <v>35.4243</v>
       </c>
     </row>
     <row r="148">
@@ -27348,7 +27348,7 @@
         <v>0</v>
       </c>
       <c r="H153" t="n">
-        <v>40.2685</v>
+        <v>40.2684</v>
       </c>
     </row>
     <row r="154">
@@ -27457,7 +27457,7 @@
         <v>0</v>
       </c>
       <c r="G157" t="n">
-        <v>50.6737</v>
+        <v>50.6736</v>
       </c>
       <c r="H157" t="n">
         <v>0</v>
@@ -27513,7 +27513,7 @@
         <v>0</v>
       </c>
       <c r="G159" t="n">
-        <v>59.7734</v>
+        <v>59.7733</v>
       </c>
       <c r="H159" t="n">
         <v>0</v>
@@ -27541,7 +27541,7 @@
         <v>0</v>
       </c>
       <c r="G160" t="n">
-        <v>74.6972</v>
+        <v>74.69710000000001</v>
       </c>
       <c r="H160" t="n">
         <v>0</v>
@@ -27569,7 +27569,7 @@
         <v>0</v>
       </c>
       <c r="G161" t="n">
-        <v>45.6432</v>
+        <v>45.6431</v>
       </c>
       <c r="H161" t="n">
         <v>0</v>
@@ -27625,7 +27625,7 @@
         <v>0</v>
       </c>
       <c r="G163" t="n">
-        <v>55.5997</v>
+        <v>55.5996</v>
       </c>
       <c r="H163" t="n">
         <v>0</v>
@@ -28297,7 +28297,7 @@
         <v>0</v>
       </c>
       <c r="G187" t="n">
-        <v>54.1502</v>
+        <v>54.1501</v>
       </c>
       <c r="H187" t="n">
         <v>0</v>
@@ -28341,7 +28341,7 @@
         <v>0</v>
       </c>
       <c r="C189" t="n">
-        <v>42.1658</v>
+        <v>42.1657</v>
       </c>
       <c r="D189" t="n">
         <v>0</v>
@@ -28372,7 +28372,7 @@
         <v>0</v>
       </c>
       <c r="D190" t="n">
-        <v>17.1528</v>
+        <v>17.1527</v>
       </c>
       <c r="E190" t="n">
         <v>0</v>
@@ -28409,7 +28409,7 @@
         <v>0</v>
       </c>
       <c r="G191" t="n">
-        <v>92.2925</v>
+        <v>92.2924</v>
       </c>
       <c r="H191" t="n">
         <v>0</v>
@@ -28661,7 +28661,7 @@
         <v>0</v>
       </c>
       <c r="G200" t="n">
-        <v>33.3876</v>
+        <v>33.3875</v>
       </c>
       <c r="H200" t="n">
         <v>0</v>
@@ -28720,7 +28720,7 @@
         <v>53.6935</v>
       </c>
       <c r="H202" t="n">
-        <v>45.8065</v>
+        <v>45.8064</v>
       </c>
     </row>
     <row r="203">
@@ -28776,7 +28776,7 @@
         <v>0</v>
       </c>
       <c r="H204" t="n">
-        <v>81.6794</v>
+        <v>81.6793</v>
       </c>
     </row>
     <row r="205">
@@ -28829,7 +28829,7 @@
         <v>0</v>
       </c>
       <c r="G206" t="n">
-        <v>47.0973</v>
+        <v>47.0972</v>
       </c>
       <c r="H206" t="n">
         <v>52.4027</v>
@@ -28944,7 +28944,7 @@
         <v>84.00700000000001</v>
       </c>
       <c r="H210" t="n">
-        <v>15.493</v>
+        <v>15.4929</v>
       </c>
     </row>
     <row r="211">
@@ -28972,7 +28972,7 @@
         <v>0</v>
       </c>
       <c r="H211" t="n">
-        <v>67.5676</v>
+        <v>67.5675</v>
       </c>
     </row>
     <row r="212">
@@ -29000,7 +29000,7 @@
         <v>0</v>
       </c>
       <c r="H212" t="n">
-        <v>72.41379999999999</v>
+        <v>72.41370000000001</v>
       </c>
     </row>
     <row r="213">
@@ -29084,7 +29084,7 @@
         <v>0</v>
       </c>
       <c r="H215" t="n">
-        <v>50.4505</v>
+        <v>50.4504</v>
       </c>
     </row>
     <row r="216">
@@ -29112,7 +29112,7 @@
         <v>0</v>
       </c>
       <c r="H216" t="n">
-        <v>20.6897</v>
+        <v>20.6896</v>
       </c>
     </row>
     <row r="217">
@@ -29140,7 +29140,7 @@
         <v>39.4449</v>
       </c>
       <c r="H217" t="n">
-        <v>60.0551</v>
+        <v>60.055</v>
       </c>
     </row>
     <row r="218">
@@ -29168,7 +29168,7 @@
         <v>42.6599</v>
       </c>
       <c r="H218" t="n">
-        <v>56.8401</v>
+        <v>56.84</v>
       </c>
     </row>
     <row r="219">
@@ -29196,7 +29196,7 @@
         <v>64.66849999999999</v>
       </c>
       <c r="H219" t="n">
-        <v>34.8315</v>
+        <v>34.8314</v>
       </c>
     </row>
     <row r="220">
@@ -29224,7 +29224,7 @@
         <v>0</v>
       </c>
       <c r="H220" t="n">
-        <v>33.5404</v>
+        <v>33.5403</v>
       </c>
     </row>
     <row r="221">
@@ -29364,7 +29364,7 @@
         <v>0</v>
       </c>
       <c r="H225" t="n">
-        <v>15.7895</v>
+        <v>15.7894</v>
       </c>
     </row>
     <row r="226">
@@ -29392,7 +29392,7 @@
         <v>0</v>
       </c>
       <c r="H226" t="n">
-        <v>20.8054</v>
+        <v>20.8053</v>
       </c>
     </row>
     <row r="227">
@@ -29445,7 +29445,7 @@
         <v>0</v>
       </c>
       <c r="G228" t="n">
-        <v>94.2149</v>
+        <v>94.2148</v>
       </c>
       <c r="H228" t="n">
         <v>0</v>
@@ -29504,7 +29504,7 @@
         <v>0</v>
       </c>
       <c r="H230" t="n">
-        <v>52.1277</v>
+        <v>52.1276</v>
       </c>
     </row>
     <row r="231">
@@ -29557,7 +29557,7 @@
         <v>0</v>
       </c>
       <c r="G232" t="n">
-        <v>81.8322</v>
+        <v>81.8321</v>
       </c>
       <c r="H232" t="n">
         <v>17.6678</v>
@@ -29672,7 +29672,7 @@
         <v>0</v>
       </c>
       <c r="H236" t="n">
-        <v>19.4631</v>
+        <v>19.463</v>
       </c>
     </row>
     <row r="237">
@@ -29756,7 +29756,7 @@
         <v>0</v>
       </c>
       <c r="H239" t="n">
-        <v>16.7702</v>
+        <v>16.7701</v>
       </c>
     </row>
     <row r="240">
@@ -30008,7 +30008,7 @@
         <v>56.4713</v>
       </c>
       <c r="H248" t="n">
-        <v>43.0287</v>
+        <v>43.0286</v>
       </c>
     </row>
     <row r="249">
@@ -30033,7 +30033,7 @@
         <v>0</v>
       </c>
       <c r="G249" t="n">
-        <v>75.1549</v>
+        <v>75.15479999999999</v>
       </c>
       <c r="H249" t="n">
         <v>24.3451</v>
@@ -30092,7 +30092,7 @@
         <v>0</v>
       </c>
       <c r="H251" t="n">
-        <v>34.2466</v>
+        <v>34.2465</v>
       </c>
     </row>
     <row r="252">
@@ -30232,7 +30232,7 @@
         <v>0</v>
       </c>
       <c r="H256" t="n">
-        <v>42.4658</v>
+        <v>42.4657</v>
       </c>
     </row>
     <row r="257">
@@ -30288,7 +30288,7 @@
         <v>57.9932</v>
       </c>
       <c r="H258" t="n">
-        <v>41.5068</v>
+        <v>41.5067</v>
       </c>
     </row>
     <row r="259">
@@ -30313,7 +30313,7 @@
         <v>0</v>
       </c>
       <c r="G259" t="n">
-        <v>65.4513</v>
+        <v>65.4512</v>
       </c>
       <c r="H259" t="n">
         <v>34.0487</v>
@@ -30512,7 +30512,7 @@
         <v>0</v>
       </c>
       <c r="H266" t="n">
-        <v>25.1799</v>
+        <v>25.1798</v>
       </c>
     </row>
     <row r="267">
@@ -30565,7 +30565,7 @@
         <v>0</v>
       </c>
       <c r="G268" t="n">
-        <v>53.1341</v>
+        <v>53.134</v>
       </c>
       <c r="H268" t="n">
         <v>46.3659</v>
@@ -30596,7 +30596,7 @@
         <v>0</v>
       </c>
       <c r="H269" t="n">
-        <v>55.4645</v>
+        <v>55.4644</v>
       </c>
     </row>
     <row r="270">
@@ -30652,7 +30652,7 @@
         <v>0</v>
       </c>
       <c r="H271" t="n">
-        <v>34.5133</v>
+        <v>34.5132</v>
       </c>
     </row>
     <row r="272">
@@ -30736,7 +30736,7 @@
         <v>0</v>
       </c>
       <c r="H274" t="n">
-        <v>27.6786</v>
+        <v>27.6785</v>
       </c>
     </row>
     <row r="275">
@@ -30848,7 +30848,7 @@
         <v>0</v>
       </c>
       <c r="H278" t="n">
-        <v>12.7451</v>
+        <v>12.745</v>
       </c>
     </row>
     <row r="279">
@@ -30929,7 +30929,7 @@
         <v>0</v>
       </c>
       <c r="G281" t="n">
-        <v>18.2796</v>
+        <v>18.2795</v>
       </c>
       <c r="H281" t="n">
         <v>0</v>
@@ -30957,7 +30957,7 @@
         <v>0</v>
       </c>
       <c r="G282" t="n">
-        <v>60.8674</v>
+        <v>60.8673</v>
       </c>
       <c r="H282" t="n">
         <v>38.6326</v>
@@ -31100,7 +31100,7 @@
         <v>0</v>
       </c>
       <c r="H287" t="n">
-        <v>27.6786</v>
+        <v>27.6785</v>
       </c>
     </row>
     <row r="288">
@@ -31240,7 +31240,7 @@
         <v>0</v>
       </c>
       <c r="H292" t="n">
-        <v>40.1961</v>
+        <v>40.196</v>
       </c>
     </row>
     <row r="293">
@@ -31309,7 +31309,7 @@
         <v>0</v>
       </c>
       <c r="C295" t="n">
-        <v>44.8229</v>
+        <v>44.8228</v>
       </c>
       <c r="D295" t="n">
         <v>0</v>
@@ -31405,7 +31405,7 @@
         <v>0</v>
       </c>
       <c r="G298" t="n">
-        <v>60.8169</v>
+        <v>60.8168</v>
       </c>
       <c r="H298" t="n">
         <v>38.6831</v>
@@ -31433,7 +31433,7 @@
         <v>0</v>
       </c>
       <c r="G299" t="n">
-        <v>85.59739999999999</v>
+        <v>85.5973</v>
       </c>
       <c r="H299" t="n">
         <v>0</v>
@@ -31461,7 +31461,7 @@
         <v>0</v>
       </c>
       <c r="G300" t="n">
-        <v>28.0229</v>
+        <v>28.0228</v>
       </c>
       <c r="H300" t="n">
         <v>0</v>
@@ -31520,7 +31520,7 @@
         <v>0</v>
       </c>
       <c r="H302" t="n">
-        <v>80.86960000000001</v>
+        <v>80.8695</v>
       </c>
     </row>
     <row r="303">
@@ -31548,7 +31548,7 @@
         <v>0</v>
       </c>
       <c r="H303" t="n">
-        <v>91.1765</v>
+        <v>91.1764</v>
       </c>
     </row>
     <row r="304">
@@ -31576,7 +31576,7 @@
         <v>0</v>
       </c>
       <c r="H304" t="n">
-        <v>94.68089999999999</v>
+        <v>94.6808</v>
       </c>
     </row>
     <row r="305">
@@ -31713,7 +31713,7 @@
         <v>0</v>
       </c>
       <c r="G309" t="n">
-        <v>58.0678</v>
+        <v>58.0677</v>
       </c>
       <c r="H309" t="n">
         <v>41.4322</v>
@@ -31825,7 +31825,7 @@
         <v>0</v>
       </c>
       <c r="G313" t="n">
-        <v>67.9358</v>
+        <v>67.9357</v>
       </c>
       <c r="H313" t="n">
         <v>31.5642</v>
@@ -31912,7 +31912,7 @@
         <v>0</v>
       </c>
       <c r="H316" t="n">
-        <v>30.4348</v>
+        <v>30.4347</v>
       </c>
     </row>
     <row r="317">
@@ -31940,7 +31940,7 @@
         <v>0</v>
       </c>
       <c r="H317" t="n">
-        <v>41.7476</v>
+        <v>41.7475</v>
       </c>
     </row>
     <row r="318">
@@ -31968,7 +31968,7 @@
         <v>0</v>
       </c>
       <c r="H318" t="n">
-        <v>28.4211</v>
+        <v>28.421</v>
       </c>
     </row>
     <row r="319">
@@ -32024,7 +32024,7 @@
         <v>0</v>
       </c>
       <c r="H320" t="n">
-        <v>39.4737</v>
+        <v>39.4736</v>
       </c>
     </row>
     <row r="321">
@@ -32052,7 +32052,7 @@
         <v>62.1301</v>
       </c>
       <c r="H321" t="n">
-        <v>37.3699</v>
+        <v>37.3698</v>
       </c>
     </row>
     <row r="322">
@@ -32108,7 +32108,7 @@
         <v>0</v>
       </c>
       <c r="H323" t="n">
-        <v>30.6667</v>
+        <v>30.6666</v>
       </c>
     </row>
     <row r="324">
@@ -32164,7 +32164,7 @@
         <v>0</v>
       </c>
       <c r="H325" t="n">
-        <v>28.0992</v>
+        <v>28.0991</v>
       </c>
     </row>
     <row r="326">
@@ -32444,7 +32444,7 @@
         <v>0</v>
       </c>
       <c r="H335" t="n">
-        <v>28.0702</v>
+        <v>28.0701</v>
       </c>
     </row>
     <row r="336">
@@ -32500,7 +32500,7 @@
         <v>0</v>
       </c>
       <c r="H337" t="n">
-        <v>43.2836</v>
+        <v>43.2835</v>
       </c>
     </row>
     <row r="338">
@@ -32665,7 +32665,7 @@
         <v>0</v>
       </c>
       <c r="G343" t="n">
-        <v>92.5926</v>
+        <v>92.5925</v>
       </c>
       <c r="H343" t="n">
         <v>0</v>
@@ -32752,7 +32752,7 @@
         <v>0</v>
       </c>
       <c r="H346" t="n">
-        <v>32.948</v>
+        <v>32.9479</v>
       </c>
     </row>
     <row r="347">
@@ -32836,7 +32836,7 @@
         <v>0</v>
       </c>
       <c r="H349" t="n">
-        <v>21.0938</v>
+        <v>21.0937</v>
       </c>
     </row>
     <row r="350">
@@ -32864,7 +32864,7 @@
         <v>0</v>
       </c>
       <c r="H350" t="n">
-        <v>23.3871</v>
+        <v>23.387</v>
       </c>
     </row>
     <row r="351">
@@ -32892,7 +32892,7 @@
         <v>0</v>
       </c>
       <c r="H351" t="n">
-        <v>27.8689</v>
+        <v>27.8688</v>
       </c>
     </row>
     <row r="352">
@@ -33116,7 +33116,7 @@
         <v>0</v>
       </c>
       <c r="H359" t="n">
-        <v>50.4762</v>
+        <v>50.4761</v>
       </c>
     </row>
     <row r="360">
@@ -33144,7 +33144,7 @@
         <v>56.7708</v>
       </c>
       <c r="H360" t="n">
-        <v>42.7292</v>
+        <v>42.7291</v>
       </c>
     </row>
     <row r="361">
@@ -33228,7 +33228,7 @@
         <v>0</v>
       </c>
       <c r="H363" t="n">
-        <v>40.3509</v>
+        <v>40.3508</v>
       </c>
     </row>
     <row r="364">
@@ -33253,7 +33253,7 @@
         <v>0</v>
       </c>
       <c r="G364" t="n">
-        <v>54.0455</v>
+        <v>54.0454</v>
       </c>
       <c r="H364" t="n">
         <v>45.4545</v>
@@ -33284,7 +33284,7 @@
         <v>0</v>
       </c>
       <c r="H365" t="n">
-        <v>64.7059</v>
+        <v>64.7058</v>
       </c>
     </row>
     <row r="366">
@@ -33340,7 +33340,7 @@
         <v>0</v>
       </c>
       <c r="H367" t="n">
-        <v>42.9719</v>
+        <v>42.9718</v>
       </c>
     </row>
     <row r="368">
@@ -33421,7 +33421,7 @@
         <v>0</v>
       </c>
       <c r="G370" t="n">
-        <v>46.6761</v>
+        <v>46.676</v>
       </c>
       <c r="H370" t="n">
         <v>52.8239</v>
@@ -33480,7 +33480,7 @@
         <v>0</v>
       </c>
       <c r="H372" t="n">
-        <v>80.6283</v>
+        <v>80.62820000000001</v>
       </c>
     </row>
     <row r="373">
@@ -33508,7 +33508,7 @@
         <v>58.1111</v>
       </c>
       <c r="H373" t="n">
-        <v>41.3889</v>
+        <v>41.3888</v>
       </c>
     </row>
     <row r="374">
@@ -33732,7 +33732,7 @@
         <v>50.2667</v>
       </c>
       <c r="H381" t="n">
-        <v>49.2333</v>
+        <v>49.2332</v>
       </c>
     </row>
     <row r="382">
@@ -33760,7 +33760,7 @@
         <v>60.8647</v>
       </c>
       <c r="H382" t="n">
-        <v>38.6353</v>
+        <v>38.6352</v>
       </c>
     </row>
     <row r="383">
@@ -33869,7 +33869,7 @@
         <v>0</v>
       </c>
       <c r="G386" t="n">
-        <v>45.8563</v>
+        <v>45.8562</v>
       </c>
       <c r="H386" t="n">
         <v>53.6437</v>
@@ -33928,7 +33928,7 @@
         <v>0</v>
       </c>
       <c r="H388" t="n">
-        <v>41.7722</v>
+        <v>41.7721</v>
       </c>
     </row>
     <row r="389">
@@ -34012,7 +34012,7 @@
         <v>0</v>
       </c>
       <c r="H391" t="n">
-        <v>48.1928</v>
+        <v>48.1927</v>
       </c>
     </row>
     <row r="392">
@@ -34152,7 +34152,7 @@
         <v>0</v>
       </c>
       <c r="H396" t="n">
-        <v>25.2033</v>
+        <v>25.2032</v>
       </c>
     </row>
     <row r="397">
@@ -34208,7 +34208,7 @@
         <v>0</v>
       </c>
       <c r="H398" t="n">
-        <v>36.9048</v>
+        <v>36.9047</v>
       </c>
     </row>
     <row r="399">
@@ -34236,7 +34236,7 @@
         <v>0</v>
       </c>
       <c r="H399" t="n">
-        <v>53.4247</v>
+        <v>53.4246</v>
       </c>
     </row>
     <row r="400">
@@ -34264,7 +34264,7 @@
         <v>0</v>
       </c>
       <c r="H400" t="n">
-        <v>46.9697</v>
+        <v>46.9696</v>
       </c>
     </row>
     <row r="401">
@@ -34289,7 +34289,7 @@
         <v>0</v>
       </c>
       <c r="G401" t="n">
-        <v>60.9286</v>
+        <v>60.9285</v>
       </c>
       <c r="H401" t="n">
         <v>38.5714</v>
@@ -34404,7 +34404,7 @@
         <v>0</v>
       </c>
       <c r="H405" t="n">
-        <v>97.29730000000001</v>
+        <v>97.2972</v>
       </c>
     </row>
     <row r="406">
@@ -34460,7 +34460,7 @@
         <v>41.768</v>
       </c>
       <c r="H407" t="n">
-        <v>57.732</v>
+        <v>57.7319</v>
       </c>
     </row>
     <row r="408">
@@ -34516,7 +34516,7 @@
         <v>0</v>
       </c>
       <c r="H409" t="n">
-        <v>80.9524</v>
+        <v>80.95229999999999</v>
       </c>
     </row>
     <row r="410">
@@ -34572,7 +34572,7 @@
         <v>69.98050000000001</v>
       </c>
       <c r="H411" t="n">
-        <v>29.5195</v>
+        <v>29.5194</v>
       </c>
     </row>
     <row r="412">
@@ -34992,7 +34992,7 @@
         <v>0</v>
       </c>
       <c r="H426" t="n">
-        <v>98.6014</v>
+        <v>98.60129999999999</v>
       </c>
     </row>
     <row r="427">
@@ -35020,7 +35020,7 @@
         <v>0</v>
       </c>
       <c r="H427" t="n">
-        <v>44.8485</v>
+        <v>44.8484</v>
       </c>
     </row>
     <row r="428">
@@ -35272,7 +35272,7 @@
         <v>0</v>
       </c>
       <c r="H436" t="n">
-        <v>57.5758</v>
+        <v>57.5757</v>
       </c>
     </row>
     <row r="437">
@@ -35300,7 +35300,7 @@
         <v>0</v>
       </c>
       <c r="H437" t="n">
-        <v>60.8696</v>
+        <v>60.8695</v>
       </c>
     </row>
     <row r="438">
@@ -35356,7 +35356,7 @@
         <v>0</v>
       </c>
       <c r="H439" t="n">
-        <v>43.6508</v>
+        <v>43.6507</v>
       </c>
     </row>
     <row r="440">
@@ -35384,7 +35384,7 @@
         <v>0</v>
       </c>
       <c r="H440" t="n">
-        <v>60.1399</v>
+        <v>60.1398</v>
       </c>
     </row>
     <row r="441">
@@ -35468,7 +35468,7 @@
         <v>0</v>
       </c>
       <c r="H443" t="n">
-        <v>44.6809</v>
+        <v>44.6808</v>
       </c>
     </row>
     <row r="444">
@@ -35720,7 +35720,7 @@
         <v>0</v>
       </c>
       <c r="H452" t="n">
-        <v>45.8537</v>
+        <v>45.8536</v>
       </c>
     </row>
     <row r="453">
@@ -35860,7 +35860,7 @@
         <v>0</v>
       </c>
       <c r="H457" t="n">
-        <v>40.678</v>
+        <v>40.6779</v>
       </c>
     </row>
     <row r="458">
@@ -36000,7 +36000,7 @@
         <v>73.3019</v>
       </c>
       <c r="H462" t="n">
-        <v>26.1981</v>
+        <v>26.198</v>
       </c>
     </row>
     <row r="463">
@@ -36053,7 +36053,7 @@
         <v>0</v>
       </c>
       <c r="G464" t="n">
-        <v>46.6642</v>
+        <v>46.6641</v>
       </c>
       <c r="H464" t="n">
         <v>52.8358</v>
@@ -36196,7 +36196,7 @@
         <v>0</v>
       </c>
       <c r="H469" t="n">
-        <v>94.2029</v>
+        <v>94.2028</v>
       </c>
     </row>
     <row r="470">
@@ -36361,7 +36361,7 @@
         <v>0</v>
       </c>
       <c r="G475" t="n">
-        <v>51.9814</v>
+        <v>51.9813</v>
       </c>
       <c r="H475" t="n">
         <v>0</v>
@@ -36476,7 +36476,7 @@
         <v>0</v>
       </c>
       <c r="H479" t="n">
-        <v>38.5455</v>
+        <v>38.5454</v>
       </c>
     </row>
     <row r="480">
@@ -36756,7 +36756,7 @@
         <v>0</v>
       </c>
       <c r="H489" t="n">
-        <v>22.449</v>
+        <v>22.4489</v>
       </c>
     </row>
     <row r="490">
@@ -36784,7 +36784,7 @@
         <v>0</v>
       </c>
       <c r="H490" t="n">
-        <v>42.069</v>
+        <v>42.0689</v>
       </c>
     </row>
     <row r="491">
@@ -36840,7 +36840,7 @@
         <v>0</v>
       </c>
       <c r="H492" t="n">
-        <v>38.3459</v>
+        <v>38.3458</v>
       </c>
     </row>
     <row r="493">
@@ -36868,7 +36868,7 @@
         <v>0</v>
       </c>
       <c r="H493" t="n">
-        <v>62.0513</v>
+        <v>62.0512</v>
       </c>
     </row>
     <row r="494">
@@ -36896,7 +36896,7 @@
         <v>0</v>
       </c>
       <c r="H494" t="n">
-        <v>43.8017</v>
+        <v>43.8016</v>
       </c>
     </row>
     <row r="495">
@@ -36952,7 +36952,7 @@
         <v>0</v>
       </c>
       <c r="H496" t="n">
-        <v>48.855</v>
+        <v>48.8549</v>
       </c>
     </row>
     <row r="497">
@@ -37120,7 +37120,7 @@
         <v>0</v>
       </c>
       <c r="H502" t="n">
-        <v>37.8049</v>
+        <v>37.8048</v>
       </c>
     </row>
     <row r="503">
@@ -37484,7 +37484,7 @@
         <v>0</v>
       </c>
       <c r="H515" t="n">
-        <v>44.6154</v>
+        <v>44.6153</v>
       </c>
     </row>
     <row r="516">
@@ -37680,7 +37680,7 @@
         <v>0</v>
       </c>
       <c r="H522" t="n">
-        <v>29.0323</v>
+        <v>29.0322</v>
       </c>
     </row>
     <row r="523">
@@ -37708,7 +37708,7 @@
         <v>0</v>
       </c>
       <c r="H523" t="n">
-        <v>26.3441</v>
+        <v>26.344</v>
       </c>
     </row>
     <row r="524">
@@ -37736,7 +37736,7 @@
         <v>0</v>
       </c>
       <c r="H524" t="n">
-        <v>22.5131</v>
+        <v>22.513</v>
       </c>
     </row>
     <row r="525">
@@ -37792,7 +37792,7 @@
         <v>0</v>
       </c>
       <c r="H526" t="n">
-        <v>41.6667</v>
+        <v>41.6666</v>
       </c>
     </row>
     <row r="527">
@@ -37848,7 +37848,7 @@
         <v>0</v>
       </c>
       <c r="H528" t="n">
-        <v>35.1852</v>
+        <v>35.1851</v>
       </c>
     </row>
     <row r="529">
@@ -37876,7 +37876,7 @@
         <v>0</v>
       </c>
       <c r="H529" t="n">
-        <v>37.594</v>
+        <v>37.5939</v>
       </c>
     </row>
     <row r="530">
@@ -37904,7 +37904,7 @@
         <v>0</v>
       </c>
       <c r="H530" t="n">
-        <v>35.533</v>
+        <v>35.5329</v>
       </c>
     </row>
     <row r="531">
@@ -37932,7 +37932,7 @@
         <v>0</v>
       </c>
       <c r="H531" t="n">
-        <v>19.697</v>
+        <v>19.6969</v>
       </c>
     </row>
     <row r="532">
@@ -37988,7 +37988,7 @@
         <v>0</v>
       </c>
       <c r="H533" t="n">
-        <v>46.7662</v>
+        <v>46.7661</v>
       </c>
     </row>
     <row r="534">
@@ -38100,7 +38100,7 @@
         <v>0</v>
       </c>
       <c r="H537" t="n">
-        <v>30.8725</v>
+        <v>30.8724</v>
       </c>
     </row>
     <row r="538">
@@ -38209,7 +38209,7 @@
         <v>0</v>
       </c>
       <c r="G541" t="n">
-        <v>72.68819999999999</v>
+        <v>72.68810000000001</v>
       </c>
       <c r="H541" t="n">
         <v>0</v>
@@ -38349,7 +38349,7 @@
         <v>0</v>
       </c>
       <c r="G546" t="n">
-        <v>71.1844</v>
+        <v>71.18429999999999</v>
       </c>
       <c r="H546" t="n">
         <v>0</v>
@@ -38377,7 +38377,7 @@
         <v>0</v>
       </c>
       <c r="G547" t="n">
-        <v>88.7427</v>
+        <v>88.7426</v>
       </c>
       <c r="H547" t="n">
         <v>0</v>
@@ -38405,7 +38405,7 @@
         <v>0</v>
       </c>
       <c r="G548" t="n">
-        <v>37.0746</v>
+        <v>37.0745</v>
       </c>
       <c r="H548" t="n">
         <v>0</v>

</xml_diff>